<commit_message>
feat: add cell merging for first and second level menus
</commit_message>
<xml_diff>
--- a/菜单导出.xlsx
+++ b/菜单导出.xlsx
@@ -1506,6 +1506,23 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B12:B17"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B39:B53"/>
+    <mergeCell ref="A3:A53"/>
+    <mergeCell ref="B54:B62"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B72:B79"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="A72:A81"/>
+    <mergeCell ref="B22:B38"/>
+    <mergeCell ref="A54:A62"/>
+    <mergeCell ref="B7:B11"/>
+    <mergeCell ref="A63:A67"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: filter out rows without url, add left align and vertical center
</commit_message>
<xml_diff>
--- a/菜单导出.xlsx
+++ b/菜单导出.xlsx
@@ -70,13 +70,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.796875" customWidth="1" min="1" max="1"/>
@@ -483,1023 +490,1002 @@
       <c r="E2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>点检管理</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>数据统计</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>全厂统计</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stat/MachStat.html</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>点检人员统计</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/PatrollerStatic.html</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>点检执行情况</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/MachineMonitor.html</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>启停机管理</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machoff/Index.html</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>标准管理</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>企标管理</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stdofmeas/QStdMgr.html</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>企标审核</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stdofmeas/QStdCheck.html</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>执行标准管理</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stdofmeas/Index.html</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>执行标准审核</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stdofmeas/CheckIndex.html</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>执行标准下发</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/stdofmeas/OneKeySetList.html</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>点检管理</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>设备浏览</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/machtree/NodeNavi.html</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>计划组态</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/plan/Index.html</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>计划下载</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/issues/Down.html</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>计划回收</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/issues/Recive.html</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>备机管理</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machoff/StandByIndex.html</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>违规管理</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/anti/Index.html</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>报警管理</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>报警查询</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/AlarmNavi.html</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>报警确认</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/alarmconfirm/UnConfirmIndex.html</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>报警审核</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/alarmconfirm/ConfirmIndex.html</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>报警阈值导入</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/threshold/AlarmThreshold.html</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>基础数据</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>设备结构树</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/machtree/Edit.html</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>设备主次管理</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machimpo/MachImpoIndex.html</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>设备等级管理</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machinelevel/MachineLevelList.html</t>
         </is>
       </c>
     </row>
     <row r="25" ht="13.9" customHeight="1">
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>设备类型管理</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machinetype/MachType.html</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>区域类型管理</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/workareatype/WorkAreaTypeList.html</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>专业类型管理</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/spectype/SpecTypeList.html</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>信号类型管理</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/signal/Index.html</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>观察量管理</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/signal/ObsMgr.html</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>仪器管理</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/collector/Index.html</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>扩展属性</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/exprop/ExPropList.html</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>轴承库管理</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/bearing/BearingList.html</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>特征频率管理</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/featurefreq/GroupList.html</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>启停机原因管理</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machoff/ReasonList.html</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>诊断助手</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/examine/Index.html</t>
         </is>
       </c>
     </row>
     <row r="36" ht="13.9" customHeight="1">
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>注释码管理</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/notecode/Index.html</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>部件类型管理</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machpartstype/MachPartsTypeList.html</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>RBD部件管理</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/partspoint/Edit.html</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>数据查询分析</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>巡检数据分析</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>~/areas/analyze/AnalyzeView.html</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>巡检数据查询</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/Patrol.html</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>波形数据查询</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/Wave.html</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>临时数据查询管理</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/TmpPatrol.html</t>
         </is>
       </c>
     </row>
     <row r="43" ht="13.9" customHeight="1">
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>电子标签未触碰</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/EmarkTouch.html</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>设备查询</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>~/areas/machbase/machine/MachQuery.html</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>位置查询</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/location/LocQuery.html</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>测点查询</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>~/areas/measure/point/PointQuery.html</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>历史数据管理</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/history/Index.html</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>动平衡报告</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/DynBalance.html</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>违规查询</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/AntiRuleQuery.html</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>计划查询</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/PlanQuery.html</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>最新巡检数据</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/LatestPatrol.html</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>注释码历史数据</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/HistoryNoteCodeIndex.html</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>漏检计划查询</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/query/UndetectedPlan.html</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>运维管理</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>缺陷管理</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>缺陷导航</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/index.html</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>缺陷总览</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/allview.html</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>缺陷新增</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/Edit.html</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>缺陷确认</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/ListDefectConfirm.html</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>缺陷分派</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/ListDefectAllot.html</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>缺陷反馈</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/listfeedback.html</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>缺陷验证</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/listreformcheck.html</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>缺陷查询</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/defectquery.html</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>缺陷补录</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t>~/areas/defecttrace/defect/defectrecord.html</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>状态监测</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>实时监控</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>设备浏览</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/machtree/NodeNavi.html</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>分析诊断</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>诊断助手</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>~/areas/inspect/examine/Index.html</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>数据挖掘</t>
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>文档管理</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>文档管理</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>文件浏览</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/docsystem/folder/BrowseIndex.html</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>往复机械故障定位</t>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>文件管理</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/docsystem/folder/Index.html</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>在线监测组态</t>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>文件夹类型管理</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/docsystem/foldertype/Index.html</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>文档管理</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>文档管理</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>文件浏览</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>~/areas/docsystem/folder/BrowseIndex.html</t>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>文件类型管理</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/docsystem/filetype/Index.html</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>文件管理</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>~/areas/docsystem/folder/Index.html</t>
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>后台管理</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>基础数据</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>部门管理</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/department/Index.html</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>文件夹类型管理</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>~/areas/docsystem/foldertype/Index.html</t>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>菜单配置</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/syscfg/menucfg.html</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>文件类型管理</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>~/areas/docsystem/filetype/Index.html</t>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>用户管理</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/user/Index.html</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>后台管理</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>基础数据</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>部门管理</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/department/Index.html</t>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>角色管理</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/role/Index.html</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>菜单配置</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/syscfg/menucfg.html</t>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>操作权限点</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/syscfg/FuncList.html</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>用户管理</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/user/Index.html</t>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>操作权限配置</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/syscfg/PermissionList.html</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>角色管理</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/role/Index.html</t>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>操作名称管理</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/syscfg/OperateList.html</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>操作权限点</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/syscfg/FuncList.html</t>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>节点权限管理</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/machbase/usermachineaccess/Index.html</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>操作权限配置</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/syscfg/PermissionList.html</t>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>系统日志</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>操作日志管理</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>~/areas/sysbase/operatelog/Index.html</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>操作名称管理</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/syscfg/OperateList.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>节点权限管理</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>~/areas/machbase/usermachineaccess/Index.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>系统日志</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>操作日志管理</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>~/areas/sysbase/operatelog/Index.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>系统配置</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>文档管理系统配置</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>~/areas/docsystem/setting/Index.html</t>
         </is>
@@ -1508,20 +1494,20 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="B12:B17"/>
+    <mergeCell ref="B69:B76"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A65:A68"/>
     <mergeCell ref="B39:B53"/>
     <mergeCell ref="A3:A53"/>
     <mergeCell ref="B54:B62"/>
     <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B72:B79"/>
     <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="A72:A81"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A69:A78"/>
     <mergeCell ref="B22:B38"/>
     <mergeCell ref="A54:A62"/>
     <mergeCell ref="B7:B11"/>
-    <mergeCell ref="A63:A67"/>
+    <mergeCell ref="B65:B68"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>